<commit_message>
Mapeo de los casos recuperacion de clave 38529 y OTP 38526
</commit_message>
<xml_diff>
--- a/control/Control_Ejecucion.xlsx
+++ b/control/Control_Ejecucion.xlsx
@@ -1879,24 +1879,72 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38529 - Recuperacion de clave con CC</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REC-001</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SI</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AUTO</t>
+        </is>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recuperacion de clave: cambia la clave de un cliente registrado del listado</t>
+        </is>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38526 - OTP en la recuperacion de clave</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REC-OTP-001</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SI</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AUTO</t>
+        </is>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OTP en la recuperacion de clave (mismo escenario de 38529)</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
@@ -6753,7 +6801,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Caso no valido" error="Seleccione un caso de la lista (casos construidos)." xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
-            <xm:f>Catalogo!$A$2:$A$12</xm:f>
+            <xm:f>Catalogo!$A$2:$A$14</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A500</xm:sqref>
         </x14:dataValidation>
@@ -7111,10 +7159,16 @@
       <c r="H11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="J11" s="4"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Disponible en la hoja Control (REC-OTP-001). Mismo escenario de 38529; el evento del OTP no se ve en la app (verificacion fuera de la UI). En la app el OTP se pide despues de la clave nueva</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:10" ht="210" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
@@ -7141,11 +7195,15 @@
       <c r="H12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>84</v>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Automatizado</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Disponible en la hoja Control (REC-001). RN-R07 confirmada. En la app la clave nueva se pide antes del OTP</t>
+        </is>
       </c>
     </row>
     <row r="13" spans="1:10" ht="255" x14ac:dyDescent="0.25">
@@ -7807,7 +7865,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -8050,6 +8108,70 @@
         <v>242</v>
       </c>
     </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38529 - Recuperacion de clave con CC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38529</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recuperacion de clave</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@38529</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TipoDocumento (CC)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NumDocumento: AUTO o vacio toma un cliente REGISTRADO con clave del listado (sin LINEA_SMS). Clave = la nueva: vacia se genera segun RN-R07 y distinta de la actual; si se informa debe cumplir RN-R07. OTP: vacio = 000000. Cambia la clave del cliente: el listado guarda la nueva al confirmar; si falla tras enviar el cambio queda FALLIDO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38526 - OTP en la recuperacion de clave</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38526</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recuperacion de clave</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@38526</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TipoDocumento (CC)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mismo escenario y reglas de 38529 (el OTP es un paso del flujo de recuperacion). El evento "Recuperacion de contrasena" del OTP no se ve en la app: se verifica fuera de la UI.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>